<commit_message>
feat: introduce new data file for IPP analysis and enhance validation notebook with additional calculations and execution count adjustments; update output files for improved results representation
</commit_message>
<xml_diff>
--- a/studies/ipp/outputs/ipp_validation_results.xlsx
+++ b/studies/ipp/outputs/ipp_validation_results.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -447,7 +447,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.994421171219982</v>
+        <v>0.997278653142597</v>
       </c>
     </row>
     <row r="3">
@@ -457,7 +457,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.9920990006674331</v>
+        <v>0.9960661441300729</v>
       </c>
     </row>
     <row r="4">
@@ -467,7 +467,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.9756400561844274</v>
+        <v>0.9890606556575989</v>
       </c>
     </row>
     <row r="5">
@@ -477,7 +477,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.9942939503873636</v>
+        <v>0.9977375893947902</v>
       </c>
     </row>
     <row r="6">
@@ -487,7 +487,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.9929724749318315</v>
+        <v>0.9961859406795989</v>
       </c>
     </row>
     <row r="7">
@@ -497,7 +497,67 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.9778746496190258</v>
+        <v>0.9915048351925559</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Cronbach's Alpha (Full Scale)</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0.7628513423860002</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Cronbach's Alpha (Especialização)</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0.5556000388486964</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Cronbach's Alpha (Carreira)</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0.6554042590733344</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>McDonald's Omega (Especialização)</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0.6221965294132332</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>McDonald's Omega (Carreira)</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0.7852265639986714</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>McDonald's Omega Total (2-factor)</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.8281967676932912</v>
       </c>
     </row>
   </sheetData>

</xml_diff>